<commit_message>
Add latest template.xlsx file
</commit_message>
<xml_diff>
--- a/luke_wip/Template.xlsx
+++ b/luke_wip/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\luke\SwimifyHandler\luke_wip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31FCC56-1E44-4FEE-82C5-6EA187123BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB5966E-E8D3-4344-8302-0D7A3A89CAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31080" yWindow="3660" windowWidth="28800" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="4" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="400m" sheetId="8" r:id="rId6"/>
     <sheet name="800m" sheetId="9" r:id="rId7"/>
     <sheet name="1500m" sheetId="10" r:id="rId8"/>
+    <sheet name="PB" sheetId="13" r:id="rId9"/>
   </sheets>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="53">
   <si>
     <t>slut-tid</t>
   </si>
@@ -259,7 +260,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -452,6 +453,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -528,7 +538,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -612,6 +622,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="73">
@@ -2811,4 +2827,43 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C60123C-9B6E-4E71-A60B-EE9C21915AD6}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="3" width="6.875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="7" style="3" customWidth="1"/>
+    <col min="7" max="7" width="7.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="9.625" style="1" customWidth="1"/>
+    <col min="14" max="17" width="10.625" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>